<commit_message>
Added RAD ContinueButton and Negative SSN test cases
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/UM-Data.xlsx
+++ b/KatalonData/Bootstrap/UM-Data.xlsx
@@ -1,45 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{7B68E34D-93B4-40FB-B2DA-4965D8FF65C5}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A4D584-EFA5-4D3A-B60C-08722AB64BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="5" firstSheet="3" windowHeight="16776" windowWidth="30936" xWindow="45972" xr2:uid="{354FC140-4496-4D7F-AB69-566E59F6C646}" yWindow="2952"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="3" activeTab="5" xr2:uid="{354FC140-4496-4D7F-AB69-566E59F6C646}"/>
   </bookViews>
   <sheets>
-    <sheet name="CreateUser" r:id="rId1" sheetId="1"/>
-    <sheet name="CreateUserSpCharError" r:id="rId2" sheetId="2"/>
-    <sheet name="CreateUserSCFNameErr" r:id="rId3" sheetId="9"/>
-    <sheet name="CreateUserSCLNameErr" r:id="rId4" sheetId="10"/>
-    <sheet name="CreateUserSpChar" r:id="rId5" sheetId="3"/>
-    <sheet name="UsernameCase" r:id="rId6" sheetId="5"/>
-    <sheet name="UsernameCaseDemo" r:id="rId7" sheetId="21"/>
-    <sheet name="PassCase" r:id="rId8" sheetId="6"/>
-    <sheet name="PassCaseDemo" r:id="rId9" sheetId="20"/>
-    <sheet name="FindUser" r:id="rId10" sheetId="7"/>
-    <sheet name="FindUserDemo" r:id="rId11" sheetId="18"/>
-    <sheet name="CreateUserErrors" r:id="rId12" sheetId="8"/>
-    <sheet name="TestForTyler" r:id="rId13" sheetId="11"/>
-    <sheet name="TestLogin" r:id="rId14" sheetId="12"/>
-    <sheet name="CreateUserPasswordSpChar" r:id="rId15" sheetId="13"/>
-    <sheet name="ModifyUser" r:id="rId16" sheetId="14"/>
-    <sheet name="ModifyUserPwd" r:id="rId17" sheetId="15"/>
-    <sheet name="ModifyUserPwdDemo" r:id="rId18" sheetId="19"/>
-    <sheet name="AddDeleteRole" r:id="rId19" sheetId="16"/>
-    <sheet name="SearchRole" r:id="rId20" sheetId="17"/>
+    <sheet name="CreateUser" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateUserSpCharError" sheetId="2" r:id="rId2"/>
+    <sheet name="CreateUserSCFNameErr" sheetId="9" r:id="rId3"/>
+    <sheet name="CreateUserSCLNameErr" sheetId="10" r:id="rId4"/>
+    <sheet name="CreateUserSpChar" sheetId="3" r:id="rId5"/>
+    <sheet name="UsernameCase" sheetId="5" r:id="rId6"/>
+    <sheet name="UsernameCaseDemo" sheetId="21" r:id="rId7"/>
+    <sheet name="PassCase" sheetId="6" r:id="rId8"/>
+    <sheet name="PassCaseDemo" sheetId="20" r:id="rId9"/>
+    <sheet name="FindUser" sheetId="7" r:id="rId10"/>
+    <sheet name="FindUserDemo" sheetId="18" r:id="rId11"/>
+    <sheet name="CreateUserErrors" sheetId="8" r:id="rId12"/>
+    <sheet name="TestForTyler" sheetId="11" r:id="rId13"/>
+    <sheet name="TestLogin" sheetId="12" r:id="rId14"/>
+    <sheet name="CreateUserPasswordSpChar" sheetId="13" r:id="rId15"/>
+    <sheet name="ModifyUser" sheetId="14" r:id="rId16"/>
+    <sheet name="ModifyUserPwd" sheetId="15" r:id="rId17"/>
+    <sheet name="ModifyUserPwdDemo" sheetId="19" r:id="rId18"/>
+    <sheet name="AddDeleteRole" sheetId="16" r:id="rId19"/>
+    <sheet name="SearchRole" sheetId="17" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="12" name="_xlnm._FilterDatabase">TestForTyler!$A$1:$A$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">TestForTyler!$A$1:$A$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="275">
   <si>
     <t>Result</t>
   </si>
@@ -611,18 +611,6 @@
     <t>Sat Aug 16 21:39:55 EDT 2025</t>
   </si>
   <si>
-    <t>Sat Nov 15 18:26:12 EST 2025</t>
-  </si>
-  <si>
-    <t>Sat Nov 15 18:26:59 EST 2025</t>
-  </si>
-  <si>
-    <t>Sat Nov 15 18:27:48 EST 2025</t>
-  </si>
-  <si>
-    <t>Sat Nov 15 18:28:36 EST 2025</t>
-  </si>
-  <si>
     <t>Sat Nov 15 18:29:24 EST 2025</t>
   </si>
   <si>
@@ -773,36 +761,6 @@
     <t>chraguis2</t>
   </si>
   <si>
-    <t>Fri Feb 20 19:33:33 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:33:52 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:34:16 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:34:39 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:34:59 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:35:18 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:35:37 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:35:56 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:36:16 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:41:15 EST 2026</t>
-  </si>
-  <si>
     <t>chraguis</t>
   </si>
   <si>
@@ -812,12 +770,6 @@
     <t>Fri Feb 20 20:07:30 EST 2026</t>
   </si>
   <si>
-    <t>Fri Feb 20 20:08:22 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 20:08:43 EST 2026</t>
-  </si>
-  <si>
     <t>Fri Feb 20 20:40:55 EST 2026</t>
   </si>
   <si>
@@ -881,12 +833,6 @@
     <t>Tue Jun 02 18:07:56 EDT 2026</t>
   </si>
   <si>
-    <t>Hello@3333333</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>Thu Jun 04 16:14:58 EDT 2026</t>
   </si>
   <si>
@@ -933,13 +879,15 @@
   </si>
   <si>
     <t>Thu Jun 04 16:35:04 EDT 2026</t>
+  </si>
+  <si>
+    <t>Hello@4444444</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -996,28 +944,28 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
-    <xf applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="2" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="1" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="1"/>
-    <xf applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0"/>
-    <xf applyFill="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle builtinId="8" name="Hyperlink" xfId="1"/>
-    <cellStyle builtinId="0" name="Normal" xfId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1034,10 +982,10 @@
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1072,7 +1020,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin panose="020F0302020204030204" typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1124,7 +1072,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin panose="020F0502020204030204" typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1235,21 +1183,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="6350">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1266,7 +1214,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1318,29 +1266,29 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" name="Office 2013 - 2022 Theme" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E041308-6561-4EE5-9DD4-5DDA2695E487}">
-  <dimension ref="A1:L4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E041308-6561-4EE5-9DD4-5DDA2695E487}">
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="14.19921875" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="1" width="9.796875" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="1" width="9.46484375" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" style="1" width="23.53125" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="29.19921875" collapsed="true"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="1" width="4.796875" collapsed="true"/>
-    <col min="12" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="26.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="14.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="9.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="9.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="26.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="23.53125" style="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="29.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="4.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
@@ -1383,7 +1331,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -1409,7 +1357,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -1435,7 +1383,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -1457,8 +1405,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -1466,19 +1414,19 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D7D96D8-F32A-42CB-8719-B4A22D28EC0D}">
-  <dimension ref="A1:I13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D7D96D8-F32A-42CB-8719-B4A22D28EC0D}">
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="19.46484375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="25.796875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="1" width="10.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="13.796875" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="1" width="14.73046875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="1" width="11.46484375" collapsed="true"/>
-    <col min="9" max="16384" style="1" width="19.46484375" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="25.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="10" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="13.796875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="14.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="11.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="16384" width="19.46484375" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
@@ -1512,13 +1460,13 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>27</v>
@@ -1529,7 +1477,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -1546,7 +1494,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -1563,7 +1511,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>283</v>
+        <v>265</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -1580,7 +1528,7 @@
         <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
@@ -1597,7 +1545,7 @@
         <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>285</v>
+        <v>267</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -1614,7 +1562,7 @@
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
@@ -1631,7 +1579,7 @@
         <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
@@ -1648,7 +1596,7 @@
         <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
@@ -1665,7 +1613,7 @@
         <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>11</v>
@@ -1682,7 +1630,7 @@
         <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>290</v>
+        <v>272</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
@@ -1699,7 +1647,7 @@
         <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>291</v>
+        <v>273</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>11</v>
@@ -1712,8 +1660,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -1721,18 +1669,18 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34901AB0-515C-47DD-9878-C056CC0F5D3B}">
-  <dimension ref="A1:I13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34901AB0-515C-47DD-9878-C056CC0F5D3B}">
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="23.86328125" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="5.33203125" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="6.86328125" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="8.73046875" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" width="13.3984375" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" width="12.265625" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" width="18.796875" collapsed="true"/>
+    <col min="1" max="1" width="5.59765625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="23.86328125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="8.73046875" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="13.3984375" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="12.265625" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="18.796875" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
@@ -1766,14 +1714,14 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1786,7 +1734,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
@@ -1942,28 +1890,28 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93BF1DC6-8140-4BB0-A2E7-1959BCD7413E}">
-  <dimension ref="A1:M17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93BF1DC6-8140-4BB0-A2E7-1959BCD7413E}">
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultColWidth="47.53125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="14.33203125" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="18.265625" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="19.796875" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="1" width="20.53125" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="1" width="23.796875" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" style="1" width="36.0" collapsed="true"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" style="1" width="35.46484375" collapsed="true"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="1" width="4.796875" collapsed="true"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="1" width="45.53125" collapsed="true"/>
-    <col min="13" max="16384" style="1" width="47.53125" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="26.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="14.33203125" style="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="18.265625" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="19.796875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="20.53125" style="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="23.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="36" style="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="35.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="4.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="12" width="45.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="13" max="16384" width="47.53125" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
@@ -2009,7 +1957,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -2044,7 +1992,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -2079,7 +2027,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -2114,7 +2062,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -2149,7 +2097,7 @@
         <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
@@ -2179,7 +2127,7 @@
         <v>149</v>
       </c>
     </row>
-    <row ht="28.5" r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -2219,7 +2167,7 @@
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>11</v>
@@ -2254,7 +2202,7 @@
         <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
@@ -2289,7 +2237,7 @@
         <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>11</v>
@@ -2324,7 +2272,7 @@
         <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>11</v>
@@ -2359,7 +2307,7 @@
         <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
@@ -2389,7 +2337,7 @@
         <v>160</v>
       </c>
     </row>
-    <row ht="28.5" r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -2424,7 +2372,7 @@
         <v>149</v>
       </c>
     </row>
-    <row ht="28.5" r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -2471,14 +2419,14 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="I13" xr:uid="{3F9F44A8-9B34-41E9-BAB0-00A6C19D92F8}"/>
-    <hyperlink r:id="rId2" ref="I12" xr:uid="{72B34BFC-1C06-4629-A7D1-00835E578F1C}"/>
-    <hyperlink r:id="rId3" ref="J12" xr:uid="{05843862-7C41-4D97-A198-1A33D27EECAF}"/>
-    <hyperlink r:id="rId4" ref="J13" xr:uid="{4B596713-18AE-4E73-886D-498F1C2E6C62}"/>
-    <hyperlink r:id="rId5" ref="I7" xr:uid="{03AFAD0B-8C1E-4C88-9D19-59B6814BCD72}"/>
+    <hyperlink ref="I13" r:id="rId1" xr:uid="{3F9F44A8-9B34-41E9-BAB0-00A6C19D92F8}"/>
+    <hyperlink ref="I12" r:id="rId2" xr:uid="{72B34BFC-1C06-4629-A7D1-00835E578F1C}"/>
+    <hyperlink ref="J12" r:id="rId3" xr:uid="{05843862-7C41-4D97-A198-1A33D27EECAF}"/>
+    <hyperlink ref="J13" r:id="rId4" xr:uid="{4B596713-18AE-4E73-886D-498F1C2E6C62}"/>
+    <hyperlink ref="I7" r:id="rId5" xr:uid="{03AFAD0B-8C1E-4C88-9D19-59B6814BCD72}"/>
   </hyperlinks>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId6" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId6"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -2486,17 +2434,17 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D08B5C-751A-493E-80A1-F414BB27DBFB}">
-  <dimension ref="A1:G41"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D08B5C-751A-493E-80A1-F414BB27DBFB}">
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultColWidth="16.265625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.19921875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="1" width="10.0" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="1" width="10.19921875" collapsed="true"/>
-    <col min="7" max="16384" style="1" width="16.265625" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="26.19921875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="10" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="10.19921875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="16384" width="16.265625" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -3202,19 +3150,19 @@
   </sheetData>
   <autoFilter ref="A1:A41" xr:uid="{06D08B5C-751A-493E-80A1-F414BB27DBFB}"/>
   <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{448B252B-DA85-45B5-97C8-A61A3A927843}">
-  <dimension ref="A1:E31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{448B252B-DA85-45B5-97C8-A61A3A927843}">
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultColWidth="12.53125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="34.796875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="8.0" collapsed="true"/>
+    <col min="2" max="2" width="34.796875" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -3236,7 +3184,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -3562,30 +3510,30 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74BBB4B9-A457-4811-8CDB-D2D99106F229}">
-  <dimension ref="A1:N17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74BBB4B9-A457-4811-8CDB-D2D99106F229}">
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="1" width="28.0" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="38.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="21.0" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="3" width="21.265625" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="1" width="9.796875" collapsed="true"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" style="1" width="9.46484375" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="11" max="11" customWidth="true" style="1" width="15.0" collapsed="true"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="1" width="16.73046875" collapsed="true"/>
-    <col min="13" max="13" customWidth="true" style="1" width="12.73046875" collapsed="true"/>
-    <col min="14" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="28" style="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="38.265625" style="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="8" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="21" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="21.265625" style="3" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="9.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="9.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="26.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="15" style="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="12" width="16.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="13" max="13" width="12.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="14" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.45">
@@ -3629,12 +3577,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>128</v>
@@ -3650,12 +3598,12 @@
       </c>
       <c r="J2" s="2"/>
     </row>
-    <row ht="28.5" r="3" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>128</v>
@@ -3671,12 +3619,12 @@
       </c>
       <c r="J3" s="2"/>
     </row>
-    <row ht="28.5" r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>128</v>
@@ -3691,12 +3639,12 @@
         <v>9</v>
       </c>
     </row>
-    <row ht="28.5" r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>128</v>
@@ -3711,12 +3659,12 @@
         <v>9</v>
       </c>
     </row>
-    <row ht="28.5" r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>128</v>
@@ -3731,12 +3679,12 @@
         <v>9</v>
       </c>
     </row>
-    <row ht="28.5" r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>128</v>
@@ -3751,12 +3699,12 @@
         <v>9</v>
       </c>
     </row>
-    <row ht="28.5" r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>128</v>
@@ -3771,12 +3719,12 @@
         <v>9</v>
       </c>
     </row>
-    <row ht="28.5" r="9" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>128</v>
@@ -3791,12 +3739,12 @@
         <v>9</v>
       </c>
     </row>
-    <row ht="28.5" r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>128</v>
@@ -3811,12 +3759,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>128</v>
@@ -3831,12 +3779,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>128</v>
@@ -3851,12 +3799,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>128</v>
@@ -3871,12 +3819,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>128</v>
@@ -3891,12 +3839,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="15" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>53</v>
       </c>
       <c r="B15" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>128</v>
@@ -3911,12 +3859,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>53</v>
       </c>
       <c r="B16" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>128</v>
@@ -3931,12 +3879,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="28.5" r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>128</v>
@@ -3953,28 +3901,28 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B8F5FA-1070-472D-B967-69AFD2883CDC}">
-  <dimension ref="A1:L3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B8F5FA-1070-472D-B967-69AFD2883CDC}">
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="14.19921875" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" style="1" width="9.796875" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="1" width="9.46484375" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" style="1" width="23.53125" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="29.19921875" collapsed="true"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="1" width="4.796875" collapsed="true"/>
-    <col min="12" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="26.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="14.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="9.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="9.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="26.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="23.53125" style="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="29.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="4.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
@@ -4017,7 +3965,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -4043,7 +3991,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4065,24 +4013,24 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{633A7FE5-E252-4628-A48A-457CABF49F07}">
-  <dimension ref="A1:K8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{633A7FE5-E252-4628-A48A-457CABF49F07}">
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultColWidth="19.46484375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="19.46484375" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="22.53125" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="13.796875" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="1" width="14.73046875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="1" width="11.46484375" collapsed="true"/>
-    <col min="9" max="16384" style="1" width="19.46484375" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="26.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="19.46484375" style="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="22.53125" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="13.796875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="14.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="11.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="16384" width="19.46484375" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
@@ -4122,7 +4070,7 @@
         <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>169</v>
@@ -4148,7 +4096,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4265,25 +4213,25 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA21BF1A-0002-4471-AB72-BBFC45A36DFE}">
-  <dimension ref="A1:K8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA21BF1A-0002-4471-AB72-BBFC45A36DFE}">
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" width="37.59765625" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" width="16.59765625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="6.86328125" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" width="15.73046875" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="8.53125" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="8.265625" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" width="19.19921875" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" width="17.796875" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" width="20.73046875" collapsed="true"/>
+    <col min="1" max="1" width="5.59765625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="37.59765625" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="16.59765625" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="15.73046875" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="8.53125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="8.265625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="19.19921875" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="17.796875" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="20.73046875" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
@@ -4323,7 +4271,7 @@
         <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>169</v>
@@ -4332,7 +4280,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -4351,14 +4299,14 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -4378,7 +4326,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -4398,7 +4346,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -4418,7 +4366,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -4440,7 +4388,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -4460,7 +4408,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -4475,21 +4423,21 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A53983D-C89C-4548-8A02-C36CB8EC5C28}">
-  <dimension ref="A1:G5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A53983D-C89C-4548-8A02-C36CB8EC5C28}">
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="5" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="5" width="29.796875" collapsed="true"/>
-    <col min="3" max="4" style="5" width="9.19921875" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="5" width="18.46484375" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="5" width="21.0" collapsed="true"/>
-    <col min="7" max="16384" style="5" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="5" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="29.796875" style="5" customWidth="1" collapsed="1"/>
+    <col min="3" max="4" width="9.19921875" style="5" collapsed="1"/>
+    <col min="5" max="5" width="18.46484375" style="5" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="21" style="5" customWidth="1" collapsed="1"/>
+    <col min="7" max="16384" width="9.19921875" style="5" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -4517,7 +4465,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>258</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>11</v>
@@ -4534,7 +4482,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>277</v>
+        <v>259</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>11</v>
@@ -4551,7 +4499,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>278</v>
+        <v>260</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>11</v>
@@ -4568,7 +4516,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>11</v>
@@ -4581,28 +4529,28 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DB9BADB-29CB-4747-93B5-EAB1AD94407A}">
-  <dimension ref="A1:M7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DB9BADB-29CB-4747-93B5-EAB1AD94407A}">
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="25.0" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="16.796875" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="14.19921875" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="1" width="9.796875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="1" width="9.46484375" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="15.0" collapsed="true"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="1" width="16.73046875" collapsed="true"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="1" width="4.796875" collapsed="true"/>
-    <col min="13" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="25" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="16.796875" style="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="8" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="14.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="9.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="9.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="26.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="15" style="1" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="16.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="12" width="4.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="13" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
@@ -4648,7 +4596,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -4666,7 +4614,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4684,7 +4632,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -4702,7 +4650,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -4720,7 +4668,7 @@
         <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
@@ -4738,7 +4686,7 @@
         <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -4752,7 +4700,7 @@
       <c r="I7" s="2"/>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -4760,16 +4708,16 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCABF931-E9E5-40BE-B844-C9FC3C47A38B}">
-  <dimension ref="A1:G5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCABF931-E9E5-40BE-B844-C9FC3C47A38B}">
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="5" width="9.19921875" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="5" width="22.73046875" collapsed="true"/>
-    <col min="3" max="4" style="5" width="9.19921875" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="5" width="24.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="5" width="22.73046875" collapsed="true"/>
-    <col min="7" max="16384" style="5" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="9.19921875" style="5" collapsed="1"/>
+    <col min="2" max="2" width="22.73046875" style="5" customWidth="1" collapsed="1"/>
+    <col min="3" max="4" width="9.19921875" style="5" collapsed="1"/>
+    <col min="5" max="5" width="24" style="5" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="22.73046875" style="5" customWidth="1" collapsed="1"/>
+    <col min="7" max="16384" width="9.19921875" style="5" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -4797,7 +4745,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>11</v>
@@ -4814,7 +4762,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>11</v>
@@ -4831,7 +4779,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>11</v>
@@ -4848,7 +4796,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>11</v>
@@ -4861,20 +4809,20 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A029BA7-3086-406C-A77E-58AC14E2F6FE}">
-  <dimension ref="A1:F5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A029BA7-3086-406C-A77E-58AC14E2F6FE}">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="25.796875" collapsed="true"/>
-    <col min="3" max="4" style="1" width="9.19921875" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="12.19921875" collapsed="true"/>
-    <col min="6" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="9.19921875" style="1" collapsed="1"/>
+    <col min="2" max="2" width="25.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="4" width="9.19921875" style="1" collapsed="1"/>
+    <col min="5" max="5" width="12.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -4899,7 +4847,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -4913,7 +4861,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -4927,7 +4875,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -4941,7 +4889,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -4951,8 +4899,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -4960,11 +4908,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B88DB0-56A9-4751-A2AB-F86F5E9F992C}">
-  <dimension ref="A1:F5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B88DB0-56A9-4751-A2AB-F86F5E9F992C}">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="14.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="16384" style="1" width="14.796875" collapsed="true"/>
+    <col min="1" max="16384" width="14.796875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -4989,7 +4937,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5003,7 +4951,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -5017,7 +4965,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -5031,7 +4979,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -5041,8 +4989,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -5050,23 +4998,23 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B5C51F8-B59C-42E8-82FD-350399CB099A}">
-  <dimension ref="A1:M4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B5C51F8-B59C-42E8-82FD-350399CB099A}">
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="25.796875" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="16.796875" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="14.19921875" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="1" width="9.796875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="1" width="9.46484375" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" style="1" width="26.73046875" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="15.0" collapsed="true"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" style="1" width="16.73046875" collapsed="true"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" style="1" width="4.796875" collapsed="true"/>
-    <col min="13" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="25.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="16.796875" style="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="8" style="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="14.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="9.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="9.46484375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="26.73046875" style="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="15" style="1" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="16.73046875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="12" width="4.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="13" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
@@ -5112,7 +5060,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5130,7 +5078,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -5148,7 +5096,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -5161,7 +5109,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -5169,17 +5117,17 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92052058-09B3-4B5F-984B-5ED260F80AB1}">
-  <dimension ref="A1:G4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92052058-09B3-4B5F-984B-5ED260F80AB1}">
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="25.796875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="1" width="10.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="22.19921875" collapsed="true"/>
-    <col min="7" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="25.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="10" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="22.19921875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -5207,7 +5155,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>264</v>
+        <v>248</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5224,7 +5172,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -5241,7 +5189,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
@@ -5254,8 +5202,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -5263,16 +5211,16 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09030ED-B1B6-4055-8EEA-622399DA2F68}">
-  <dimension ref="A1:G4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09030ED-B1B6-4055-8EEA-622399DA2F68}">
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="23.86328125" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="5.33203125" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="6.86328125" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" width="16.796875" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" width="26.796875" collapsed="true"/>
+    <col min="1" max="1" width="5.59765625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="23.86328125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="16.796875" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="26.796875" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -5300,17 +5248,17 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
@@ -5318,17 +5266,17 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>261</v>
+        <v>245</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -5336,41 +5284,41 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>262</v>
+        <v>246</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="F2" xr:uid="{8B296A81-C701-4567-9B0A-7C1146022B98}"/>
-    <hyperlink r:id="rId2" ref="F3" xr:uid="{DC4C87CF-8300-4771-8426-123B72F2B005}"/>
-    <hyperlink r:id="rId3" ref="F4" xr:uid="{F65EAC6E-F220-4E3B-B09A-3DADF6E5F450}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{8B296A81-C701-4567-9B0A-7C1146022B98}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{DC4C87CF-8300-4771-8426-123B72F2B005}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{F65EAC6E-F220-4E3B-B09A-3DADF6E5F450}"/>
   </hyperlinks>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B91231D0-74A2-4955-BD46-A8F29393EF1C}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B91231D0-74A2-4955-BD46-A8F29393EF1C}">
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="6.53125" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="25.796875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="6.265625" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="8.0" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" style="1" width="10.0" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="14.796875" collapsed="true"/>
-    <col min="7" max="16384" style="1" width="9.19921875" collapsed="true"/>
+    <col min="1" max="1" width="6.53125" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="25.796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="6.265625" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="10" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="14.796875" style="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="16384" width="9.19921875" style="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -5398,7 +5346,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>260</v>
+        <v>244</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -5411,8 +5359,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup horizontalDpi="4294967293" orientation="portrait" r:id="rId1" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -5420,12 +5368,12 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08922CF9-D8C9-40D7-83B1-B55281F5C6AE}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08922CF9-D8C9-40D7-83B1-B55281F5C6AE}">
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="18.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.53125" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" width="8.46484375" collapsed="true"/>
+    <col min="2" max="2" width="26.53125" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="8.46484375" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -5453,14 +5401,14 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>243</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>151</v>
@@ -5468,8 +5416,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="F2" xr:uid="{C3C2FF03-5C1F-44E4-9178-C94056B18C01}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{C3C2FF03-5C1F-44E4-9178-C94056B18C01}"/>
   </hyperlinks>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>